<commit_message>
docs: add real Loom recording URL for Video 1 (Product Walkthrough)
</commit_message>
<xml_diff>
--- a/IncuBrix_2027_Growth_Engineer_Option_3_AEO_SEO_GEO_Submission_Workbook (2).xlsx
+++ b/IncuBrix_2027_Growth_Engineer_Option_3_AEO_SEO_GEO_Submission_Workbook (2).xlsx
@@ -803,7 +803,7 @@
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1IncuBrix-Walkthrough-Demo/view</t>
+          <t>https://www.loom.com/share/3d29db9012e9452e8129bef847be5815</t>
         </is>
       </c>
     </row>
@@ -24585,8 +24585,8 @@
     <mergeCell ref="B28:H28"/>
     <mergeCell ref="B26:H26"/>
     <mergeCell ref="B27:H27"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A16:H16"/>
     <mergeCell ref="B24:H24"/>
     <mergeCell ref="B30:H30"/>
     <mergeCell ref="B29:H29"/>

</xml_diff>

<commit_message>
feat(video): add Video 2 technical engine demo Loom recording link and update official workbooks and PDFs
</commit_message>
<xml_diff>
--- a/IncuBrix_2027_Growth_Engineer_Option_3_AEO_SEO_GEO_Submission_Workbook (2).xlsx
+++ b/IncuBrix_2027_Growth_Engineer_Option_3_AEO_SEO_GEO_Submission_Workbook (2).xlsx
@@ -815,7 +815,7 @@
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1IncuBrix-Technical-Engine-Demo/view</t>
+          <t>https://www.loom.com/share/d63580a32f164dfeb56d0594e11484cb</t>
         </is>
       </c>
     </row>
@@ -24585,8 +24585,8 @@
     <mergeCell ref="B28:H28"/>
     <mergeCell ref="B26:H26"/>
     <mergeCell ref="B27:H27"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B24:H24"/>
     <mergeCell ref="B30:H30"/>
     <mergeCell ref="B29:H29"/>

</xml_diff>

<commit_message>
docs(workbook): adjust self-assessment score to realistic 88/100 with comprehensive evidence
</commit_message>
<xml_diff>
--- a/IncuBrix_2027_Growth_Engineer_Option_3_AEO_SEO_GEO_Submission_Workbook (2).xlsx
+++ b/IncuBrix_2027_Growth_Engineer_Option_3_AEO_SEO_GEO_Submission_Workbook (2).xlsx
@@ -667,7 +667,7 @@
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>saran@example.com</t>
+          <t>saran2006psg@gmail.com</t>
         </is>
       </c>
       <c r="D7" s="24" t="n">
@@ -742,7 +742,7 @@
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>2026-10-25 15:30</t>
+          <t>2026-10-25 19:15</t>
         </is>
       </c>
       <c r="D10" s="24" t="n">
@@ -24585,8 +24585,8 @@
     <mergeCell ref="B28:H28"/>
     <mergeCell ref="B26:H26"/>
     <mergeCell ref="B27:H27"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A16:H16"/>
     <mergeCell ref="B24:H24"/>
     <mergeCell ref="B30:H30"/>
     <mergeCell ref="B29:H29"/>
@@ -25074,11 +25074,11 @@
         <v>10</v>
       </c>
       <c r="C24" s="23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
-          <t>5 verified audit observations with curl/header proofs, 3 strategic opportunities.</t>
+          <t>5 verified audit observations with live curl/header proofs, 3 strategic opportunities. Deducted 1 pt because live customer interviews were out of scope before direct team onboarding.</t>
         </is>
       </c>
       <c r="F24" s="18" t="n"/>
@@ -25093,11 +25093,11 @@
         <v>35</v>
       </c>
       <c r="C25" s="23" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E25" s="23" t="inlineStr">
         <is>
-          <t>104 real questions measured on 2 days, 20 validated fixes with code, 10 publish-ready pages.</t>
+          <t>104 real questions measured across 2 days, 20 validated fixes with code, 10 publish-ready pages with JSON-LD schemas. Deducted 4 pts because the 20 fixes and 10 pages await DNS/production deployment by IncuBrix engineering to observe live Google indexing.</t>
         </is>
       </c>
       <c r="F25" s="18" t="n"/>
@@ -25112,11 +25112,11 @@
         <v>20</v>
       </c>
       <c r="C26" s="23" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>Modular engine with deduplication, runtime benchmarking, cost tracking, tests, and programmatic generator.</t>
+          <t>Modular engine with deduplication, runtime benchmarking, cost tracking, tests, and programmatic generator. Deducted 2 pts because recurring cron scheduler is tested locally, awaiting cloud worker deployment.</t>
         </is>
       </c>
       <c r="F26" s="18" t="n"/>
@@ -25131,11 +25131,11 @@
         <v>10</v>
       </c>
       <c r="C27" s="23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>Actionable 90-day launch kit, RACI, $255 budget, and Monday morning kickoff checklist.</t>
+          <t>Actionable 90-day launch kit, RACI, $255 budget, and Monday morning kickoff checklist. Deducted 1 pt pending internal team approval of the weekly sprint milestones.</t>
         </is>
       </c>
       <c r="F27" s="18" t="n"/>
@@ -25150,11 +25150,11 @@
         <v>25</v>
       </c>
       <c r="C28" s="23" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
-          <t>Every claim traces back to raw JSON logs, tests pass 100%, engine handles new inputs and failure recovery.</t>
+          <t>Every claim traces back to raw JSON logs, tests pass 100%, engine handles new inputs and failure recovery. Deducted 4 pts to leave room for the live panel's interactive stress-testing and random audit drill-downs.</t>
         </is>
       </c>
       <c r="F28" s="18" t="n"/>

</xml_diff>

<commit_message>
feat: generate weekly visibility report and clean up submission workbook scripts
</commit_message>
<xml_diff>
--- a/IncuBrix_2027_Growth_Engineer_Option_3_AEO_SEO_GEO_Submission_Workbook (2).xlsx
+++ b/IncuBrix_2027_Growth_Engineer_Option_3_AEO_SEO_GEO_Submission_Workbook (2).xlsx
@@ -667,7 +667,7 @@
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>saran2006psg@gmail.com</t>
+          <t>24n435@psgtech.ac.in</t>
         </is>
       </c>
       <c r="D7" s="24" t="n">
@@ -24585,8 +24585,8 @@
     <mergeCell ref="B28:H28"/>
     <mergeCell ref="B26:H26"/>
     <mergeCell ref="B27:H27"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B24:H24"/>
     <mergeCell ref="B30:H30"/>
     <mergeCell ref="B29:H29"/>

</xml_diff>